<commit_message>
fix(docs): Update Excel schema template with missing sub-schema field guidance
* added missing description of sub-schema Parameter property usage

Refs: <sha>
Story:
Reviewed-by:
Test-scope: n

Signed-off-by: Daniel Swid <daniel.swid@hashgraph.com>
</commit_message>
<xml_diff>
--- a/guardian-service/artifacts/template.xlsx
+++ b/guardian-service/artifacts/template.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10830"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BF2B582-8F4E-BA43-8B5B-29D6D9A8B0D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CA34127-7160-3547-A282-DB9D4DA4792D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="34560" windowHeight="21600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="5" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="187">
   <si>
     <t xml:space="preserve">  Guardian Schema Template</t>
   </si>
@@ -588,6 +588,9 @@
   </si>
   <si>
     <t>Hidden field computed from other field values. Parameter must not be empty. Parameter = math expression using Test Value-cell addresses (e.g. G6 + G7). Only supported on top-level Verifiable Credential schemas (not sub-schemas).</t>
+  </si>
+  <si>
+    <t>Optional. The Parameter property is used together with the Description property to create a unique sub-schema id. This can be used to differentiate two sub-schemas with the same Description field. To reuse a sub-schema in different places, all properties of child fields must be equal.</t>
   </si>
 </sst>
 </file>
@@ -595,8 +598,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.00"/>
-    <numFmt numFmtId="169" formatCode="#,##0.00&quot;kg&quot;"/>
+    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="#,##0.00&quot;kg&quot;"/>
   </numFmts>
   <fonts count="16" x14ac:knownFonts="1">
     <font>
@@ -1197,6 +1200,132 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="13" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="15" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="15" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="14" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="14" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="15" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="15" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="14" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="14" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1208,132 +1337,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="3" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="3" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="13" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="14" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="14" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="14" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="14" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="12" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="15" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="15" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="15" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="15" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1683,800 +1686,825 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="26" x14ac:dyDescent="0.2">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="47" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
     </row>
     <row r="2" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="35" t="s">
+      <c r="A2" s="48" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="35"/>
-      <c r="C2" s="35"/>
+      <c r="B2" s="48"/>
+      <c r="C2" s="48"/>
     </row>
     <row r="3" spans="1:3" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="36"/>
-      <c r="B3" s="36"/>
-      <c r="C3" s="36"/>
+      <c r="A3" s="49"/>
+      <c r="B3" s="49"/>
+      <c r="C3" s="49"/>
     </row>
     <row r="4" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A4" s="37" t="s">
+      <c r="A4" s="36" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="37"/>
-      <c r="C4" s="37"/>
+      <c r="B4" s="36"/>
+      <c r="C4" s="36"/>
     </row>
     <row r="5" spans="1:3" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="27" t="s">
+      <c r="A5" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="27" t="s">
+      <c r="B5" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="27" t="s">
+      <c r="C5" s="23" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A6" s="28" t="s">
+      <c r="A6" s="24" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="29" t="s">
+      <c r="B6" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="29" t="s">
+      <c r="C6" s="25" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="45" x14ac:dyDescent="0.2">
-      <c r="A7" s="30" t="s">
+      <c r="A7" s="26" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="31" t="s">
+      <c r="B7" s="27" t="s">
         <v>155</v>
       </c>
-      <c r="C7" s="31" t="s">
+      <c r="C7" s="27" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="30" x14ac:dyDescent="0.2">
-      <c r="A8" s="28" t="s">
+      <c r="A8" s="24" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="29" t="s">
+      <c r="B8" s="25" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="29" t="s">
+      <c r="C8" s="25" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="38"/>
-      <c r="B9" s="38"/>
-      <c r="C9" s="38"/>
+      <c r="A9" s="35"/>
+      <c r="B9" s="35"/>
+      <c r="C9" s="35"/>
     </row>
     <row r="10" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A10" s="37" t="s">
+      <c r="A10" s="36" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="37"/>
-      <c r="C10" s="37"/>
+      <c r="B10" s="36"/>
+      <c r="C10" s="36"/>
     </row>
     <row r="11" spans="1:3" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="27" t="s">
+      <c r="A11" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="B11" s="27" t="s">
+      <c r="B11" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="C11" s="27" t="s">
+      <c r="C11" s="23" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A12" s="28" t="s">
+      <c r="A12" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="29" t="s">
+      <c r="B12" s="25" t="s">
         <v>172</v>
       </c>
-      <c r="C12" s="29"/>
+      <c r="C12" s="25"/>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A13" s="30" t="s">
+      <c r="A13" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="B13" s="31" t="s">
+      <c r="B13" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="31"/>
+      <c r="C13" s="27"/>
     </row>
     <row r="14" spans="1:3" ht="90" x14ac:dyDescent="0.2">
-      <c r="A14" s="28" t="s">
+      <c r="A14" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="B14" s="29" t="s">
+      <c r="B14" s="25" t="s">
         <v>173</v>
       </c>
-      <c r="C14" s="29" t="s">
+      <c r="C14" s="25" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="38"/>
-      <c r="B15" s="38"/>
-      <c r="C15" s="38"/>
+      <c r="A15" s="35"/>
+      <c r="B15" s="35"/>
+      <c r="C15" s="35"/>
     </row>
     <row r="16" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A16" s="37" t="s">
+      <c r="A16" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="37"/>
-      <c r="C16" s="37"/>
+      <c r="B16" s="36"/>
+      <c r="C16" s="36"/>
     </row>
     <row r="17" spans="1:3" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="27" t="s">
+      <c r="A17" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="B17" s="27" t="s">
+      <c r="B17" s="23" t="s">
         <v>22</v>
       </c>
-      <c r="C17" s="27" t="s">
+      <c r="C17" s="23" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A18" s="28" t="s">
+      <c r="A18" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="B18" s="29" t="s">
+      <c r="B18" s="25" t="s">
         <v>174</v>
       </c>
-      <c r="C18" s="29" t="s">
+      <c r="C18" s="25" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="30" x14ac:dyDescent="0.2">
-      <c r="A19" s="30" t="s">
+      <c r="A19" s="26" t="s">
         <v>25</v>
       </c>
-      <c r="B19" s="31" t="s">
+      <c r="B19" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="C19" s="31" t="s">
+      <c r="C19" s="27" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="45" x14ac:dyDescent="0.2">
-      <c r="A20" s="28" t="s">
+      <c r="A20" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="B20" s="29" t="s">
+      <c r="B20" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="C20" s="29" t="s">
+      <c r="C20" s="25" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="45" x14ac:dyDescent="0.2">
-      <c r="A21" s="30" t="s">
+      <c r="A21" s="26" t="s">
         <v>31</v>
       </c>
-      <c r="B21" s="31" t="s">
+      <c r="B21" s="27" t="s">
         <v>32</v>
       </c>
-      <c r="C21" s="31" t="s">
+      <c r="C21" s="27" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A22" s="28" t="s">
+      <c r="A22" s="24" t="s">
         <v>41</v>
       </c>
-      <c r="B22" s="29" t="s">
+      <c r="B22" s="25" t="s">
         <v>34</v>
       </c>
-      <c r="C22" s="29" t="s">
+      <c r="C22" s="25" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A23" s="30" t="s">
+      <c r="A23" s="26" t="s">
         <v>36</v>
       </c>
-      <c r="B23" s="31" t="s">
+      <c r="B23" s="27" t="s">
         <v>175</v>
       </c>
-      <c r="C23" s="31" t="s">
+      <c r="C23" s="27" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="45" x14ac:dyDescent="0.2">
-      <c r="A24" s="28" t="s">
+      <c r="A24" s="24" t="s">
         <v>165</v>
       </c>
-      <c r="B24" s="29" t="s">
+      <c r="B24" s="25" t="s">
         <v>176</v>
       </c>
-      <c r="C24" s="29" t="s">
+      <c r="C24" s="25" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A25" s="30" t="s">
+      <c r="A25" s="26" t="s">
         <v>163</v>
       </c>
-      <c r="B25" s="31" t="s">
+      <c r="B25" s="27" t="s">
         <v>178</v>
       </c>
-      <c r="C25" s="31" t="s">
+      <c r="C25" s="27" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A26" s="28" t="s">
+      <c r="A26" s="24" t="s">
         <v>164</v>
       </c>
-      <c r="B26" s="29" t="s">
+      <c r="B26" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="C26" s="29" t="s">
+      <c r="C26" s="25" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="45" x14ac:dyDescent="0.2">
-      <c r="A27" s="30" t="s">
+      <c r="A27" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="B27" s="31" t="s">
+      <c r="B27" s="27" t="s">
         <v>183</v>
       </c>
-      <c r="C27" s="31" t="s">
+      <c r="C27" s="27" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="38"/>
-      <c r="B28" s="38"/>
-      <c r="C28" s="38"/>
+      <c r="A28" s="35"/>
+      <c r="B28" s="35"/>
+      <c r="C28" s="35"/>
     </row>
     <row r="29" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A29" s="37" t="s">
+      <c r="A29" s="36" t="s">
         <v>39</v>
       </c>
-      <c r="B29" s="37"/>
-      <c r="C29" s="37"/>
+      <c r="B29" s="36"/>
+      <c r="C29" s="36"/>
     </row>
     <row r="30" spans="1:3" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="27" t="s">
+      <c r="A30" s="23" t="s">
         <v>40</v>
       </c>
-      <c r="B30" s="27" t="s">
+      <c r="B30" s="23" t="s">
         <v>41</v>
       </c>
-      <c r="C30" s="27" t="s">
+      <c r="C30" s="23" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A31" s="28" t="s">
+      <c r="A31" s="24" t="s">
         <v>43</v>
       </c>
-      <c r="B31" s="29" t="s">
+      <c r="B31" s="25" t="s">
         <v>44</v>
       </c>
-      <c r="C31" s="29" t="s">
+      <c r="C31" s="25" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A32" s="30" t="s">
+      <c r="A32" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="B32" s="31" t="s">
+      <c r="B32" s="27" t="s">
         <v>47</v>
       </c>
-      <c r="C32" s="31" t="s">
+      <c r="C32" s="27" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A33" s="28" t="s">
+      <c r="A33" s="24" t="s">
         <v>48</v>
       </c>
-      <c r="B33" s="29" t="s">
+      <c r="B33" s="25" t="s">
         <v>49</v>
       </c>
-      <c r="C33" s="29" t="s">
+      <c r="C33" s="25" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A34" s="30" t="s">
+      <c r="A34" s="26" t="s">
         <v>50</v>
       </c>
-      <c r="B34" s="31" t="s">
+      <c r="B34" s="27" t="s">
         <v>51</v>
       </c>
-      <c r="C34" s="31" t="s">
+      <c r="C34" s="27" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A35" s="28" t="s">
+      <c r="A35" s="24" t="s">
         <v>52</v>
       </c>
-      <c r="B35" s="29" t="s">
+      <c r="B35" s="25" t="s">
         <v>53</v>
       </c>
-      <c r="C35" s="29" t="s">
+      <c r="C35" s="25" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A36" s="30" t="s">
+      <c r="A36" s="26" t="s">
         <v>54</v>
       </c>
-      <c r="B36" s="31" t="s">
+      <c r="B36" s="27" t="s">
         <v>55</v>
       </c>
-      <c r="C36" s="31" t="s">
+      <c r="C36" s="27" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A37" s="28" t="s">
+      <c r="A37" s="24" t="s">
         <v>56</v>
       </c>
-      <c r="B37" s="29" t="s">
+      <c r="B37" s="25" t="s">
         <v>57</v>
       </c>
-      <c r="C37" s="29" t="s">
+      <c r="C37" s="25" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A38" s="30" t="s">
+      <c r="A38" s="26" t="s">
         <v>58</v>
       </c>
-      <c r="B38" s="31" t="s">
+      <c r="B38" s="27" t="s">
         <v>59</v>
       </c>
-      <c r="C38" s="31" t="s">
+      <c r="C38" s="27" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A39" s="28" t="s">
+      <c r="A39" s="24" t="s">
         <v>60</v>
       </c>
-      <c r="B39" s="29" t="s">
+      <c r="B39" s="25" t="s">
         <v>61</v>
       </c>
-      <c r="C39" s="29" t="s">
+      <c r="C39" s="25" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A40" s="30" t="s">
+      <c r="A40" s="26" t="s">
         <v>62</v>
       </c>
-      <c r="B40" s="31" t="s">
+      <c r="B40" s="27" t="s">
         <v>63</v>
       </c>
-      <c r="C40" s="31" t="s">
+      <c r="C40" s="27" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A41" s="28" t="s">
+      <c r="A41" s="24" t="s">
         <v>64</v>
       </c>
-      <c r="B41" s="29" t="s">
+      <c r="B41" s="25" t="s">
         <v>65</v>
       </c>
-      <c r="C41" s="29" t="s">
+      <c r="C41" s="25" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A42" s="30" t="s">
+      <c r="A42" s="26" t="s">
         <v>66</v>
       </c>
-      <c r="B42" s="31" t="s">
+      <c r="B42" s="27" t="s">
         <v>67</v>
       </c>
-      <c r="C42" s="31" t="s">
+      <c r="C42" s="27" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A43" s="28" t="s">
+      <c r="A43" s="24" t="s">
         <v>68</v>
       </c>
-      <c r="B43" s="29" t="s">
+      <c r="B43" s="25" t="s">
         <v>69</v>
       </c>
-      <c r="C43" s="29" t="s">
+      <c r="C43" s="25" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A44" s="30" t="s">
+      <c r="A44" s="26" t="s">
         <v>70</v>
       </c>
-      <c r="B44" s="31" t="s">
+      <c r="B44" s="27" t="s">
         <v>71</v>
       </c>
-      <c r="C44" s="31" t="s">
+      <c r="C44" s="27" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A45" s="28" t="s">
+      <c r="A45" s="24" t="s">
         <v>72</v>
       </c>
-      <c r="B45" s="29" t="s">
+      <c r="B45" s="25" t="s">
         <v>73</v>
       </c>
-      <c r="C45" s="29" t="s">
+      <c r="C45" s="25" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A46" s="30" t="s">
+      <c r="A46" s="26" t="s">
         <v>74</v>
       </c>
-      <c r="B46" s="31" t="s">
+      <c r="B46" s="27" t="s">
         <v>75</v>
       </c>
-      <c r="C46" s="31" t="s">
+      <c r="C46" s="27" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A47" s="28" t="s">
+      <c r="A47" s="24" t="s">
         <v>77</v>
       </c>
-      <c r="B47" s="29" t="s">
+      <c r="B47" s="25" t="s">
         <v>78</v>
       </c>
-      <c r="C47" s="29" t="s">
+      <c r="C47" s="25" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A48" s="30" t="s">
+      <c r="A48" s="26" t="s">
         <v>80</v>
       </c>
-      <c r="B48" s="31" t="s">
+      <c r="B48" s="27" t="s">
         <v>81</v>
       </c>
-      <c r="C48" s="31" t="s">
+      <c r="C48" s="27" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="49" spans="1:3" ht="60" x14ac:dyDescent="0.2">
-      <c r="A49" s="28" t="s">
+      <c r="A49" s="24" t="s">
         <v>83</v>
       </c>
-      <c r="B49" s="29" t="s">
+      <c r="B49" s="25" t="s">
         <v>179</v>
       </c>
-      <c r="C49" s="29" t="s">
+      <c r="C49" s="25" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="50" spans="1:3" ht="45" x14ac:dyDescent="0.2">
-      <c r="A50" s="30" t="s">
+    <row r="50" spans="1:3" ht="75" x14ac:dyDescent="0.2">
+      <c r="A50" s="26" t="s">
         <v>84</v>
       </c>
-      <c r="B50" s="31" t="s">
+      <c r="B50" s="27" t="s">
         <v>158</v>
       </c>
-      <c r="C50" s="31" t="s">
-        <v>45</v>
+      <c r="C50" s="27" t="s">
+        <v>186</v>
       </c>
     </row>
     <row r="51" spans="1:3" ht="75" x14ac:dyDescent="0.2">
-      <c r="A51" s="28" t="s">
+      <c r="A51" s="24" t="s">
         <v>85</v>
       </c>
-      <c r="B51" s="29" t="s">
+      <c r="B51" s="25" t="s">
         <v>185</v>
       </c>
-      <c r="C51" s="29" t="s">
+      <c r="C51" s="25" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="52" spans="1:3" ht="30" x14ac:dyDescent="0.2">
-      <c r="A52" s="30" t="s">
+      <c r="A52" s="26" t="s">
         <v>87</v>
       </c>
-      <c r="B52" s="31" t="s">
+      <c r="B52" s="27" t="s">
         <v>88</v>
       </c>
-      <c r="C52" s="31" t="s">
+      <c r="C52" s="27" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="53" spans="1:3" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="38"/>
-      <c r="B53" s="38"/>
-      <c r="C53" s="38"/>
+      <c r="A53" s="35"/>
+      <c r="B53" s="35"/>
+      <c r="C53" s="35"/>
     </row>
     <row r="54" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A54" s="37" t="s">
+      <c r="A54" s="36" t="s">
         <v>90</v>
       </c>
-      <c r="B54" s="37"/>
-      <c r="C54" s="37"/>
+      <c r="B54" s="36"/>
+      <c r="C54" s="36"/>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A55" s="32" t="s">
+      <c r="A55" s="28" t="s">
         <v>91</v>
       </c>
-      <c r="B55" s="39" t="s">
+      <c r="B55" s="45" t="s">
         <v>92</v>
       </c>
-      <c r="C55" s="40"/>
+      <c r="C55" s="46"/>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A56" s="32" t="s">
+      <c r="A56" s="28" t="s">
         <v>91</v>
       </c>
-      <c r="B56" s="41" t="s">
+      <c r="B56" s="33" t="s">
         <v>180</v>
       </c>
-      <c r="C56" s="42"/>
+      <c r="C56" s="34"/>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A57" s="32" t="s">
+      <c r="A57" s="28" t="s">
         <v>91</v>
       </c>
-      <c r="B57" s="41" t="s">
+      <c r="B57" s="33" t="s">
         <v>93</v>
       </c>
-      <c r="C57" s="42"/>
+      <c r="C57" s="34"/>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A58" s="32" t="s">
+      <c r="A58" s="28" t="s">
         <v>91</v>
       </c>
-      <c r="B58" s="41" t="s">
+      <c r="B58" s="33" t="s">
         <v>94</v>
       </c>
-      <c r="C58" s="42"/>
+      <c r="C58" s="34"/>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A59" s="32" t="s">
+      <c r="A59" s="28" t="s">
         <v>91</v>
       </c>
-      <c r="B59" s="41" t="s">
+      <c r="B59" s="33" t="s">
         <v>95</v>
       </c>
-      <c r="C59" s="42"/>
+      <c r="C59" s="34"/>
     </row>
     <row r="60" spans="1:3" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="38"/>
-      <c r="B60" s="38"/>
-      <c r="C60" s="38"/>
+      <c r="A60" s="35"/>
+      <c r="B60" s="35"/>
+      <c r="C60" s="35"/>
     </row>
     <row r="61" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A61" s="37" t="s">
+      <c r="A61" s="36" t="s">
         <v>96</v>
       </c>
-      <c r="B61" s="37"/>
-      <c r="C61" s="37"/>
+      <c r="B61" s="36"/>
+      <c r="C61" s="36"/>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A62" s="32" t="s">
+      <c r="A62" s="28" t="s">
         <v>91</v>
       </c>
-      <c r="B62" s="39" t="s">
+      <c r="B62" s="45" t="s">
         <v>97</v>
       </c>
-      <c r="C62" s="40"/>
+      <c r="C62" s="46"/>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A63" s="32" t="s">
+      <c r="A63" s="28" t="s">
         <v>91</v>
       </c>
-      <c r="B63" s="41" t="s">
+      <c r="B63" s="33" t="s">
         <v>98</v>
       </c>
-      <c r="C63" s="42"/>
+      <c r="C63" s="34"/>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A64" s="32" t="s">
+      <c r="A64" s="28" t="s">
         <v>91</v>
       </c>
-      <c r="B64" s="41" t="s">
+      <c r="B64" s="33" t="s">
         <v>99</v>
       </c>
-      <c r="C64" s="42"/>
+      <c r="C64" s="34"/>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A65" s="32" t="s">
+      <c r="A65" s="28" t="s">
         <v>91</v>
       </c>
-      <c r="B65" s="41" t="s">
+      <c r="B65" s="33" t="s">
         <v>182</v>
       </c>
-      <c r="C65" s="42"/>
+      <c r="C65" s="34"/>
     </row>
     <row r="66" spans="1:3" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="38"/>
-      <c r="B66" s="38"/>
-      <c r="C66" s="38"/>
+      <c r="A66" s="35"/>
+      <c r="B66" s="35"/>
+      <c r="C66" s="35"/>
     </row>
     <row r="67" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A67" s="37" t="s">
+      <c r="A67" s="36" t="s">
         <v>100</v>
       </c>
-      <c r="B67" s="37"/>
-      <c r="C67" s="37"/>
+      <c r="B67" s="36"/>
+      <c r="C67" s="36"/>
     </row>
     <row r="68" spans="1:3" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="27" t="s">
+      <c r="A68" s="23" t="s">
         <v>101</v>
       </c>
-      <c r="B68" s="27" t="s">
+      <c r="B68" s="23" t="s">
         <v>102</v>
       </c>
-      <c r="C68" s="27"/>
+      <c r="C68" s="23"/>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A69" s="28" t="s">
+      <c r="A69" s="24" t="s">
         <v>159</v>
       </c>
-      <c r="B69" s="29" t="s">
+      <c r="B69" s="25" t="s">
         <v>103</v>
       </c>
-      <c r="C69" s="29"/>
+      <c r="C69" s="25"/>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A70" s="30" t="s">
+      <c r="A70" s="26" t="s">
         <v>104</v>
       </c>
-      <c r="B70" s="31" t="s">
+      <c r="B70" s="27" t="s">
         <v>105</v>
       </c>
-      <c r="C70" s="31"/>
+      <c r="C70" s="27"/>
     </row>
     <row r="71" spans="1:3" ht="60" x14ac:dyDescent="0.2">
-      <c r="A71" s="30" t="s">
+      <c r="A71" s="26" t="s">
         <v>106</v>
       </c>
-      <c r="B71" s="31" t="s">
+      <c r="B71" s="27" t="s">
         <v>184</v>
       </c>
-      <c r="C71" s="31"/>
+      <c r="C71" s="27"/>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A72" s="43"/>
-      <c r="B72" s="43"/>
-      <c r="C72" s="43"/>
+      <c r="A72" s="32"/>
+      <c r="B72" s="32"/>
+      <c r="C72" s="32"/>
     </row>
     <row r="73" spans="1:3" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="27" t="s">
+      <c r="A73" s="23" t="s">
         <v>107</v>
       </c>
-      <c r="B73" s="44"/>
-      <c r="C73" s="45"/>
+      <c r="B73" s="39"/>
+      <c r="C73" s="40"/>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A74" s="32"/>
-      <c r="B74" s="46" t="s">
+      <c r="A74" s="28"/>
+      <c r="B74" s="41" t="s">
         <v>108</v>
       </c>
-      <c r="C74" s="47"/>
+      <c r="C74" s="42"/>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A75" s="32"/>
-      <c r="B75" s="48" t="s">
+      <c r="A75" s="28"/>
+      <c r="B75" s="43" t="s">
         <v>109</v>
       </c>
-      <c r="C75" s="49"/>
+      <c r="C75" s="44"/>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A76" s="32"/>
-      <c r="B76" s="48" t="s">
+      <c r="A76" s="28"/>
+      <c r="B76" s="43" t="s">
         <v>110</v>
       </c>
-      <c r="C76" s="49"/>
+      <c r="C76" s="44"/>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A77" s="32"/>
-      <c r="B77" s="48" t="s">
+      <c r="A77" s="28"/>
+      <c r="B77" s="43" t="s">
         <v>111</v>
       </c>
-      <c r="C77" s="49"/>
+      <c r="C77" s="44"/>
     </row>
     <row r="78" spans="1:3" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A78" s="38"/>
-      <c r="B78" s="38"/>
-      <c r="C78" s="38"/>
+      <c r="A78" s="35"/>
+      <c r="B78" s="35"/>
+      <c r="C78" s="35"/>
     </row>
     <row r="79" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A79" s="37" t="s">
+      <c r="A79" s="36" t="s">
         <v>177</v>
       </c>
-      <c r="B79" s="37"/>
-      <c r="C79" s="37"/>
+      <c r="B79" s="36"/>
+      <c r="C79" s="36"/>
     </row>
     <row r="80" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A80" s="33" t="s">
+      <c r="A80" s="29" t="s">
         <v>112</v>
       </c>
-      <c r="B80" s="50" t="s">
+      <c r="B80" s="37" t="s">
         <v>113</v>
       </c>
-      <c r="C80" s="51"/>
+      <c r="C80" s="38"/>
     </row>
     <row r="81" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A81" s="33" t="s">
+      <c r="A81" s="29" t="s">
         <v>112</v>
       </c>
-      <c r="B81" s="52" t="s">
+      <c r="B81" s="30" t="s">
         <v>114</v>
       </c>
-      <c r="C81" s="53"/>
+      <c r="C81" s="31"/>
     </row>
     <row r="82" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A82" s="33" t="s">
+      <c r="A82" s="29" t="s">
         <v>112</v>
       </c>
-      <c r="B82" s="52" t="s">
+      <c r="B82" s="30" t="s">
         <v>115</v>
       </c>
-      <c r="C82" s="53"/>
+      <c r="C82" s="31"/>
     </row>
     <row r="83" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A83" s="33" t="s">
+      <c r="A83" s="29" t="s">
         <v>112</v>
       </c>
-      <c r="B83" s="52" t="s">
+      <c r="B83" s="30" t="s">
         <v>116</v>
       </c>
-      <c r="C83" s="53"/>
+      <c r="C83" s="31"/>
     </row>
     <row r="84" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A84" s="33" t="s">
+      <c r="A84" s="29" t="s">
         <v>112</v>
       </c>
-      <c r="B84" s="52" t="s">
+      <c r="B84" s="30" t="s">
         <v>181</v>
       </c>
-      <c r="C84" s="53"/>
+      <c r="C84" s="31"/>
     </row>
     <row r="85" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A85" s="33" t="s">
+      <c r="A85" s="29" t="s">
         <v>112</v>
       </c>
-      <c r="B85" s="52" t="s">
+      <c r="B85" s="30" t="s">
         <v>117</v>
       </c>
-      <c r="C85" s="53"/>
+      <c r="C85" s="31"/>
     </row>
     <row r="86" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A86" s="33" t="s">
+      <c r="A86" s="29" t="s">
         <v>112</v>
       </c>
-      <c r="B86" s="52" t="s">
+      <c r="B86" s="30" t="s">
         <v>118</v>
       </c>
-      <c r="C86" s="53"/>
+      <c r="C86" s="31"/>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A87" s="43"/>
-      <c r="B87" s="43"/>
-      <c r="C87" s="43"/>
+      <c r="A87" s="32"/>
+      <c r="B87" s="32"/>
+      <c r="C87" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="41">
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="A60:C60"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="A16:C16"/>
+    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="A29:C29"/>
+    <mergeCell ref="A53:C53"/>
+    <mergeCell ref="A54:C54"/>
+    <mergeCell ref="B55:C55"/>
+    <mergeCell ref="B56:C56"/>
+    <mergeCell ref="B57:C57"/>
+    <mergeCell ref="B58:C58"/>
+    <mergeCell ref="B59:C59"/>
+    <mergeCell ref="B77:C77"/>
+    <mergeCell ref="A61:C61"/>
+    <mergeCell ref="B62:C62"/>
+    <mergeCell ref="B63:C63"/>
+    <mergeCell ref="B64:C64"/>
+    <mergeCell ref="A66:C66"/>
+    <mergeCell ref="A67:C67"/>
     <mergeCell ref="B84:C84"/>
     <mergeCell ref="B85:C85"/>
     <mergeCell ref="B86:C86"/>
@@ -2493,31 +2521,6 @@
     <mergeCell ref="B74:C74"/>
     <mergeCell ref="B75:C75"/>
     <mergeCell ref="B76:C76"/>
-    <mergeCell ref="B77:C77"/>
-    <mergeCell ref="A61:C61"/>
-    <mergeCell ref="B62:C62"/>
-    <mergeCell ref="B63:C63"/>
-    <mergeCell ref="B64:C64"/>
-    <mergeCell ref="A66:C66"/>
-    <mergeCell ref="A67:C67"/>
-    <mergeCell ref="B55:C55"/>
-    <mergeCell ref="B56:C56"/>
-    <mergeCell ref="B57:C57"/>
-    <mergeCell ref="B58:C58"/>
-    <mergeCell ref="B59:C59"/>
-    <mergeCell ref="A60:C60"/>
-    <mergeCell ref="A15:C15"/>
-    <mergeCell ref="A16:C16"/>
-    <mergeCell ref="A28:C28"/>
-    <mergeCell ref="A29:C29"/>
-    <mergeCell ref="A53:C53"/>
-    <mergeCell ref="A54:C54"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="A9:C9"/>
-    <mergeCell ref="A10:C10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -2544,50 +2547,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="51" t="s">
         <v>119</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
-      <c r="I1" s="8"/>
-      <c r="J1" s="9"/>
+      <c r="B1" s="52"/>
+      <c r="C1" s="52"/>
+      <c r="D1" s="52"/>
+      <c r="E1" s="52"/>
+      <c r="F1" s="52"/>
+      <c r="G1" s="52"/>
+      <c r="H1" s="52"/>
+      <c r="I1" s="52"/>
+      <c r="J1" s="53"/>
     </row>
     <row r="2" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="50" t="s">
         <v>120</v>
       </c>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="6"/>
-      <c r="H2" s="6"/>
-      <c r="I2" s="6"/>
-      <c r="J2" s="6"/>
+      <c r="C2" s="50"/>
+      <c r="D2" s="50"/>
+      <c r="E2" s="50"/>
+      <c r="F2" s="50"/>
+      <c r="G2" s="50"/>
+      <c r="H2" s="50"/>
+      <c r="I2" s="50"/>
+      <c r="J2" s="50"/>
     </row>
     <row r="3" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="50" t="s">
         <v>122</v>
       </c>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
-      <c r="E3" s="6"/>
-      <c r="F3" s="6"/>
-      <c r="G3" s="6"/>
-      <c r="H3" s="6"/>
-      <c r="I3" s="6"/>
-      <c r="J3" s="6"/>
+      <c r="C3" s="50"/>
+      <c r="D3" s="50"/>
+      <c r="E3" s="50"/>
+      <c r="F3" s="50"/>
+      <c r="G3" s="50"/>
+      <c r="H3" s="50"/>
+      <c r="I3" s="50"/>
+      <c r="J3" s="50"/>
     </row>
     <row r="4" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
@@ -2844,10 +2847,10 @@
       <c r="J14" s="3"/>
     </row>
     <row r="15" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A15" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="B15" s="10" t="s">
+      <c r="A15" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B15" s="6" t="s">
         <v>60</v>
       </c>
       <c r="C15" s="3"/>
@@ -2866,10 +2869,10 @@
       <c r="J15" s="3"/>
     </row>
     <row r="16" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A16" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="B16" s="10" t="s">
+      <c r="A16" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B16" s="6" t="s">
         <v>62</v>
       </c>
       <c r="C16" s="3"/>
@@ -2888,10 +2891,10 @@
       <c r="J16" s="3"/>
     </row>
     <row r="17" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A17" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="B17" s="10" t="s">
+      <c r="A17" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B17" s="6" t="s">
         <v>64</v>
       </c>
       <c r="C17" s="3"/>
@@ -2910,10 +2913,10 @@
       <c r="J17" s="3"/>
     </row>
     <row r="18" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A18" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="B18" s="10" t="s">
+      <c r="A18" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B18" s="6" t="s">
         <v>66</v>
       </c>
       <c r="C18" s="3"/>
@@ -2932,10 +2935,10 @@
       <c r="J18" s="3"/>
     </row>
     <row r="19" spans="1:10" ht="32" x14ac:dyDescent="0.2">
-      <c r="A19" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="B19" s="10" t="s">
+      <c r="A19" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B19" s="6" t="s">
         <v>87</v>
       </c>
       <c r="C19" s="3" t="s">
@@ -2954,15 +2957,15 @@
       <c r="J19" s="3"/>
     </row>
     <row r="20" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A20" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="B20" s="10" t="s">
+      <c r="A20" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B20" s="6" t="s">
         <v>70</v>
       </c>
       <c r="C20" s="3"/>
-      <c r="D20" s="11"/>
-      <c r="E20" s="10" t="s">
+      <c r="D20" s="7"/>
+      <c r="E20" s="6" t="s">
         <v>70</v>
       </c>
       <c r="F20" s="3" t="s">
@@ -2980,7 +2983,7 @@
       <c r="B21" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="C21" s="24" t="s">
+      <c r="C21" s="20" t="s">
         <v>135</v>
       </c>
       <c r="D21" s="3"/>
@@ -2990,7 +2993,7 @@
       <c r="F21" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="G21" s="25">
+      <c r="G21" s="21">
         <v>1</v>
       </c>
       <c r="H21" s="3"/>
@@ -3004,7 +3007,7 @@
       <c r="B22" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="C22" s="24" t="s">
+      <c r="C22" s="20" t="s">
         <v>137</v>
       </c>
       <c r="D22" s="3"/>
@@ -3014,7 +3017,7 @@
       <c r="F22" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="G22" s="26">
+      <c r="G22" s="22">
         <v>1</v>
       </c>
       <c r="H22" s="3"/>
@@ -3022,15 +3025,15 @@
       <c r="J22" s="3"/>
     </row>
     <row r="23" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A23" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="B23" s="10" t="s">
+      <c r="A23" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B23" s="6" t="s">
         <v>72</v>
       </c>
       <c r="C23" s="3"/>
-      <c r="D23" s="12"/>
-      <c r="E23" s="10" t="s">
+      <c r="D23" s="8"/>
+      <c r="E23" s="6" t="s">
         <v>139</v>
       </c>
       <c r="F23" s="3" t="s">
@@ -3044,21 +3047,21 @@
       <c r="J23" s="3"/>
     </row>
     <row r="24" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A24" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="B24" s="10" t="s">
+      <c r="A24" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B24" s="6" t="s">
         <v>48</v>
       </c>
       <c r="C24" s="3"/>
-      <c r="D24" s="12" t="b">
+      <c r="D24" s="8" t="b">
         <f>EXACT(G5,"Option 1")</f>
         <v>1</v>
       </c>
-      <c r="E24" s="14" t="s">
+      <c r="E24" s="10" t="s">
         <v>141</v>
       </c>
-      <c r="F24" s="10" t="s">
+      <c r="F24" s="6" t="s">
         <v>7</v>
       </c>
       <c r="G24" s="3" t="s">
@@ -3069,338 +3072,338 @@
       <c r="J24" s="3"/>
     </row>
     <row r="25" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A25" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="B25" s="14" t="s">
+      <c r="A25" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B25" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="C25" s="14"/>
-      <c r="D25" s="20" t="b">
+      <c r="C25" s="10"/>
+      <c r="D25" s="16" t="b">
         <f>NOT(EXACT(G5,"Option 1"))</f>
         <v>0</v>
       </c>
-      <c r="E25" s="14" t="s">
+      <c r="E25" s="10" t="s">
         <v>142</v>
       </c>
-      <c r="F25" s="14" t="s">
-        <v>7</v>
-      </c>
-      <c r="G25" s="14" t="s">
+      <c r="F25" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="G25" s="10" t="s">
         <v>124</v>
       </c>
-      <c r="H25" s="14"/>
-      <c r="I25" s="14"/>
-      <c r="J25" s="14"/>
+      <c r="H25" s="10"/>
+      <c r="I25" s="10"/>
+      <c r="J25" s="10"/>
     </row>
     <row r="26" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A26" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="B26" s="15" t="s">
+      <c r="A26" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B26" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="C26" s="15"/>
-      <c r="D26" s="18" t="s">
-        <v>7</v>
-      </c>
-      <c r="E26" s="15" t="s">
+      <c r="C26" s="11"/>
+      <c r="D26" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="E26" s="11" t="s">
         <v>143</v>
       </c>
-      <c r="F26" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="G26" s="15" t="s">
+      <c r="F26" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="G26" s="11" t="s">
         <v>124</v>
       </c>
-      <c r="H26" s="15"/>
-      <c r="I26" s="15"/>
-      <c r="J26" s="15"/>
+      <c r="H26" s="11"/>
+      <c r="I26" s="11"/>
+      <c r="J26" s="11"/>
     </row>
     <row r="27" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A27" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="B27" s="15" t="s">
+      <c r="A27" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B27" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="C27" s="15" t="s">
+      <c r="C27" s="11" t="s">
         <v>144</v>
       </c>
-      <c r="D27" s="18"/>
-      <c r="E27" s="15" t="s">
+      <c r="D27" s="14"/>
+      <c r="E27" s="11" t="s">
         <v>145</v>
       </c>
-      <c r="F27" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="G27" s="15">
+      <c r="F27" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="G27" s="11">
         <f>G6+G7</f>
         <v>2</v>
       </c>
-      <c r="H27" s="15"/>
-      <c r="I27" s="15"/>
-      <c r="J27" s="15"/>
+      <c r="H27" s="11"/>
+      <c r="I27" s="11"/>
+      <c r="J27" s="11"/>
     </row>
     <row r="28" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A28" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="B28" s="15" t="s">
+      <c r="A28" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B28" s="11" t="s">
         <v>84</v>
       </c>
-      <c r="C28" s="15" t="s">
+      <c r="C28" s="11" t="s">
         <v>162</v>
       </c>
-      <c r="D28" s="18"/>
-      <c r="E28" s="15" t="s">
+      <c r="D28" s="14"/>
+      <c r="E28" s="11" t="s">
         <v>168</v>
       </c>
-      <c r="F28" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="G28" s="15"/>
-      <c r="H28" s="15"/>
-      <c r="I28" s="15"/>
-      <c r="J28" s="15"/>
+      <c r="F28" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="G28" s="11"/>
+      <c r="H28" s="11"/>
+      <c r="I28" s="11"/>
+      <c r="J28" s="11"/>
     </row>
     <row r="29" spans="1:10" ht="16" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="B29" s="16" t="s">
+      <c r="A29" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B29" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="C29" s="16"/>
-      <c r="D29" s="19"/>
-      <c r="E29" s="16" t="s">
+      <c r="C29" s="12"/>
+      <c r="D29" s="15"/>
+      <c r="E29" s="12" t="s">
         <v>146</v>
       </c>
-      <c r="F29" s="16" t="s">
-        <v>7</v>
-      </c>
-      <c r="G29" s="16" t="s">
+      <c r="F29" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="G29" s="12" t="s">
         <v>147</v>
       </c>
-      <c r="H29" s="16"/>
-      <c r="I29" s="16"/>
-      <c r="J29" s="16"/>
+      <c r="H29" s="12"/>
+      <c r="I29" s="12"/>
+      <c r="J29" s="12"/>
     </row>
     <row r="30" spans="1:10" ht="16" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="13" t="s">
+      <c r="A30" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="B30" s="16" t="s">
+      <c r="B30" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="C30" s="16"/>
-      <c r="D30" s="19"/>
-      <c r="E30" s="16" t="s">
+      <c r="C30" s="12"/>
+      <c r="D30" s="15"/>
+      <c r="E30" s="12" t="s">
         <v>148</v>
       </c>
-      <c r="F30" s="16" t="s">
+      <c r="F30" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="G30" s="16">
+      <c r="G30" s="12">
         <v>1</v>
       </c>
-      <c r="H30" s="16"/>
-      <c r="I30" s="16"/>
-      <c r="J30" s="16"/>
+      <c r="H30" s="12"/>
+      <c r="I30" s="12"/>
+      <c r="J30" s="12"/>
     </row>
     <row r="31" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A31" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="B31" s="15" t="s">
+      <c r="A31" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B31" s="11" t="s">
         <v>84</v>
       </c>
-      <c r="C31" s="17" t="s">
+      <c r="C31" s="13" t="s">
         <v>162</v>
       </c>
-      <c r="D31" s="18"/>
-      <c r="E31" s="15" t="s">
+      <c r="D31" s="14"/>
+      <c r="E31" s="11" t="s">
         <v>169</v>
       </c>
-      <c r="F31" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="G31" s="15"/>
-      <c r="H31" s="15"/>
-      <c r="I31" s="15"/>
-      <c r="J31" s="15"/>
+      <c r="F31" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="G31" s="11"/>
+      <c r="H31" s="11"/>
+      <c r="I31" s="11"/>
+      <c r="J31" s="11"/>
     </row>
     <row r="32" spans="1:10" ht="16" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="B32" s="16" t="s">
+      <c r="A32" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B32" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="C32" s="16"/>
-      <c r="D32" s="19"/>
-      <c r="E32" s="16" t="s">
+      <c r="C32" s="12"/>
+      <c r="D32" s="15"/>
+      <c r="E32" s="12" t="s">
         <v>146</v>
       </c>
-      <c r="F32" s="16" t="s">
-        <v>7</v>
-      </c>
-      <c r="G32" s="16" t="s">
+      <c r="F32" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="G32" s="12" t="s">
         <v>147</v>
       </c>
-      <c r="H32" s="16"/>
-      <c r="I32" s="16"/>
-      <c r="J32" s="16"/>
+      <c r="H32" s="12"/>
+      <c r="I32" s="12"/>
+      <c r="J32" s="12"/>
     </row>
     <row r="33" spans="1:10" ht="16" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="13" t="s">
+      <c r="A33" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="B33" s="16" t="s">
+      <c r="B33" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="C33" s="16"/>
-      <c r="D33" s="19"/>
-      <c r="E33" s="16" t="s">
+      <c r="C33" s="12"/>
+      <c r="D33" s="15"/>
+      <c r="E33" s="12" t="s">
         <v>148</v>
       </c>
-      <c r="F33" s="16" t="s">
+      <c r="F33" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="G33" s="16">
+      <c r="G33" s="12">
         <v>1</v>
       </c>
-      <c r="H33" s="16"/>
-      <c r="I33" s="16"/>
-      <c r="J33" s="16"/>
+      <c r="H33" s="12"/>
+      <c r="I33" s="12"/>
+      <c r="J33" s="12"/>
     </row>
     <row r="34" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A34" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="B34" s="15" t="s">
+      <c r="A34" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B34" s="11" t="s">
         <v>84</v>
       </c>
-      <c r="C34" s="17" t="s">
+      <c r="C34" s="13" t="s">
         <v>161</v>
       </c>
-      <c r="D34" s="18"/>
-      <c r="E34" s="15" t="s">
+      <c r="D34" s="14"/>
+      <c r="E34" s="11" t="s">
         <v>170</v>
       </c>
-      <c r="F34" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="G34" s="15"/>
-      <c r="H34" s="15"/>
-      <c r="I34" s="15"/>
-      <c r="J34" s="15"/>
+      <c r="F34" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="G34" s="11"/>
+      <c r="H34" s="11"/>
+      <c r="I34" s="11"/>
+      <c r="J34" s="11"/>
     </row>
     <row r="35" spans="1:10" ht="16" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="B35" s="16" t="s">
+      <c r="A35" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B35" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="C35" s="16"/>
-      <c r="D35" s="19"/>
-      <c r="E35" s="16" t="s">
+      <c r="C35" s="12"/>
+      <c r="D35" s="15"/>
+      <c r="E35" s="12" t="s">
         <v>146</v>
       </c>
-      <c r="F35" s="16" t="s">
-        <v>7</v>
-      </c>
-      <c r="G35" s="16" t="s">
+      <c r="F35" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="G35" s="12" t="s">
         <v>147</v>
       </c>
-      <c r="H35" s="16"/>
-      <c r="I35" s="16"/>
-      <c r="J35" s="16"/>
+      <c r="H35" s="12"/>
+      <c r="I35" s="12"/>
+      <c r="J35" s="12"/>
     </row>
     <row r="36" spans="1:10" ht="16" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="19" t="s">
+      <c r="A36" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="B36" s="16" t="s">
+      <c r="B36" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="C36" s="16"/>
-      <c r="D36" s="19"/>
-      <c r="E36" s="16" t="s">
+      <c r="C36" s="12"/>
+      <c r="D36" s="15"/>
+      <c r="E36" s="12" t="s">
         <v>166</v>
       </c>
-      <c r="F36" s="16"/>
-      <c r="G36" s="16"/>
-      <c r="H36" s="16"/>
-      <c r="I36" s="16"/>
-      <c r="J36" s="16"/>
+      <c r="F36" s="12"/>
+      <c r="G36" s="12"/>
+      <c r="H36" s="12"/>
+      <c r="I36" s="12"/>
+      <c r="J36" s="12"/>
     </row>
     <row r="37" spans="1:10" ht="16" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="B37" s="15" t="s">
+      <c r="A37" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B37" s="11" t="s">
         <v>84</v>
       </c>
-      <c r="C37" s="17" t="s">
+      <c r="C37" s="13" t="s">
         <v>162</v>
       </c>
-      <c r="D37" s="18"/>
-      <c r="E37" s="15" t="s">
+      <c r="D37" s="14"/>
+      <c r="E37" s="11" t="s">
         <v>171</v>
       </c>
-      <c r="F37" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="G37" s="15"/>
-      <c r="H37" s="15"/>
-      <c r="I37" s="15"/>
-      <c r="J37" s="15"/>
+      <c r="F37" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="G37" s="11"/>
+      <c r="H37" s="11"/>
+      <c r="I37" s="11"/>
+      <c r="J37" s="11"/>
     </row>
     <row r="38" spans="1:10" ht="16" outlineLevel="2" x14ac:dyDescent="0.2">
-      <c r="A38" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="B38" s="16" t="s">
+      <c r="A38" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B38" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="C38" s="16"/>
-      <c r="D38" s="19"/>
-      <c r="E38" s="16" t="s">
+      <c r="C38" s="12"/>
+      <c r="D38" s="15"/>
+      <c r="E38" s="12" t="s">
         <v>146</v>
       </c>
-      <c r="F38" s="16" t="s">
-        <v>7</v>
-      </c>
-      <c r="G38" s="16" t="s">
+      <c r="F38" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="G38" s="12" t="s">
         <v>147</v>
       </c>
-      <c r="H38" s="16"/>
-      <c r="I38" s="16"/>
-      <c r="J38" s="16"/>
+      <c r="H38" s="12"/>
+      <c r="I38" s="12"/>
+      <c r="J38" s="12"/>
     </row>
     <row r="39" spans="1:10" ht="16" outlineLevel="2" x14ac:dyDescent="0.2">
-      <c r="A39" s="21" t="s">
+      <c r="A39" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="B39" s="22" t="s">
+      <c r="B39" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="C39" s="22"/>
-      <c r="D39" s="23"/>
-      <c r="E39" s="22" t="s">
+      <c r="C39" s="18"/>
+      <c r="D39" s="19"/>
+      <c r="E39" s="18" t="s">
         <v>148</v>
       </c>
-      <c r="F39" s="22" t="s">
+      <c r="F39" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="G39" s="22">
+      <c r="G39" s="18">
         <v>1</v>
       </c>
-      <c r="H39" s="22"/>
-      <c r="I39" s="22"/>
-      <c r="J39" s="22"/>
+      <c r="H39" s="18"/>
+      <c r="I39" s="18"/>
+      <c r="J39" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>

<commit_message>
fix(docs): Update Excel schema template with missing sub-schema field guidance (#6877)
* added missing description of sub-schema Parameter property usage

Refs: <sha>
Story:
Reviewed-by:
Test-scope: n

Signed-off-by: Daniel Swid <daniel.swid@hashgraph.com>
</commit_message>
<xml_diff>
--- a/guardian-service/artifacts/template.xlsx
+++ b/guardian-service/artifacts/template.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10830"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BF2B582-8F4E-BA43-8B5B-29D6D9A8B0D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CA34127-7160-3547-A282-DB9D4DA4792D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="34560" windowHeight="21600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="5" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="187">
   <si>
     <t xml:space="preserve">  Guardian Schema Template</t>
   </si>
@@ -588,6 +588,9 @@
   </si>
   <si>
     <t>Hidden field computed from other field values. Parameter must not be empty. Parameter = math expression using Test Value-cell addresses (e.g. G6 + G7). Only supported on top-level Verifiable Credential schemas (not sub-schemas).</t>
+  </si>
+  <si>
+    <t>Optional. The Parameter property is used together with the Description property to create a unique sub-schema id. This can be used to differentiate two sub-schemas with the same Description field. To reuse a sub-schema in different places, all properties of child fields must be equal.</t>
   </si>
 </sst>
 </file>
@@ -595,8 +598,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.00"/>
-    <numFmt numFmtId="169" formatCode="#,##0.00&quot;kg&quot;"/>
+    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="#,##0.00&quot;kg&quot;"/>
   </numFmts>
   <fonts count="16" x14ac:knownFonts="1">
     <font>
@@ -1197,6 +1200,132 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="13" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="15" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="15" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="14" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="14" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="15" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="15" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="14" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="14" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1208,132 +1337,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="3" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="3" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="13" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="14" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="14" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="14" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="14" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="12" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="15" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="15" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="15" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="15" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1683,800 +1686,825 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="26" x14ac:dyDescent="0.2">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="47" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
     </row>
     <row r="2" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="35" t="s">
+      <c r="A2" s="48" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="35"/>
-      <c r="C2" s="35"/>
+      <c r="B2" s="48"/>
+      <c r="C2" s="48"/>
     </row>
     <row r="3" spans="1:3" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="36"/>
-      <c r="B3" s="36"/>
-      <c r="C3" s="36"/>
+      <c r="A3" s="49"/>
+      <c r="B3" s="49"/>
+      <c r="C3" s="49"/>
     </row>
     <row r="4" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A4" s="37" t="s">
+      <c r="A4" s="36" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="37"/>
-      <c r="C4" s="37"/>
+      <c r="B4" s="36"/>
+      <c r="C4" s="36"/>
     </row>
     <row r="5" spans="1:3" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="27" t="s">
+      <c r="A5" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="27" t="s">
+      <c r="B5" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="27" t="s">
+      <c r="C5" s="23" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A6" s="28" t="s">
+      <c r="A6" s="24" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="29" t="s">
+      <c r="B6" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="29" t="s">
+      <c r="C6" s="25" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="45" x14ac:dyDescent="0.2">
-      <c r="A7" s="30" t="s">
+      <c r="A7" s="26" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="31" t="s">
+      <c r="B7" s="27" t="s">
         <v>155</v>
       </c>
-      <c r="C7" s="31" t="s">
+      <c r="C7" s="27" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="30" x14ac:dyDescent="0.2">
-      <c r="A8" s="28" t="s">
+      <c r="A8" s="24" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="29" t="s">
+      <c r="B8" s="25" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="29" t="s">
+      <c r="C8" s="25" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="38"/>
-      <c r="B9" s="38"/>
-      <c r="C9" s="38"/>
+      <c r="A9" s="35"/>
+      <c r="B9" s="35"/>
+      <c r="C9" s="35"/>
     </row>
     <row r="10" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A10" s="37" t="s">
+      <c r="A10" s="36" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="37"/>
-      <c r="C10" s="37"/>
+      <c r="B10" s="36"/>
+      <c r="C10" s="36"/>
     </row>
     <row r="11" spans="1:3" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="27" t="s">
+      <c r="A11" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="B11" s="27" t="s">
+      <c r="B11" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="C11" s="27" t="s">
+      <c r="C11" s="23" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A12" s="28" t="s">
+      <c r="A12" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="29" t="s">
+      <c r="B12" s="25" t="s">
         <v>172</v>
       </c>
-      <c r="C12" s="29"/>
+      <c r="C12" s="25"/>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A13" s="30" t="s">
+      <c r="A13" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="B13" s="31" t="s">
+      <c r="B13" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="31"/>
+      <c r="C13" s="27"/>
     </row>
     <row r="14" spans="1:3" ht="90" x14ac:dyDescent="0.2">
-      <c r="A14" s="28" t="s">
+      <c r="A14" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="B14" s="29" t="s">
+      <c r="B14" s="25" t="s">
         <v>173</v>
       </c>
-      <c r="C14" s="29" t="s">
+      <c r="C14" s="25" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="38"/>
-      <c r="B15" s="38"/>
-      <c r="C15" s="38"/>
+      <c r="A15" s="35"/>
+      <c r="B15" s="35"/>
+      <c r="C15" s="35"/>
     </row>
     <row r="16" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A16" s="37" t="s">
+      <c r="A16" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="37"/>
-      <c r="C16" s="37"/>
+      <c r="B16" s="36"/>
+      <c r="C16" s="36"/>
     </row>
     <row r="17" spans="1:3" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="27" t="s">
+      <c r="A17" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="B17" s="27" t="s">
+      <c r="B17" s="23" t="s">
         <v>22</v>
       </c>
-      <c r="C17" s="27" t="s">
+      <c r="C17" s="23" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A18" s="28" t="s">
+      <c r="A18" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="B18" s="29" t="s">
+      <c r="B18" s="25" t="s">
         <v>174</v>
       </c>
-      <c r="C18" s="29" t="s">
+      <c r="C18" s="25" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="30" x14ac:dyDescent="0.2">
-      <c r="A19" s="30" t="s">
+      <c r="A19" s="26" t="s">
         <v>25</v>
       </c>
-      <c r="B19" s="31" t="s">
+      <c r="B19" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="C19" s="31" t="s">
+      <c r="C19" s="27" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="45" x14ac:dyDescent="0.2">
-      <c r="A20" s="28" t="s">
+      <c r="A20" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="B20" s="29" t="s">
+      <c r="B20" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="C20" s="29" t="s">
+      <c r="C20" s="25" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="45" x14ac:dyDescent="0.2">
-      <c r="A21" s="30" t="s">
+      <c r="A21" s="26" t="s">
         <v>31</v>
       </c>
-      <c r="B21" s="31" t="s">
+      <c r="B21" s="27" t="s">
         <v>32</v>
       </c>
-      <c r="C21" s="31" t="s">
+      <c r="C21" s="27" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A22" s="28" t="s">
+      <c r="A22" s="24" t="s">
         <v>41</v>
       </c>
-      <c r="B22" s="29" t="s">
+      <c r="B22" s="25" t="s">
         <v>34</v>
       </c>
-      <c r="C22" s="29" t="s">
+      <c r="C22" s="25" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A23" s="30" t="s">
+      <c r="A23" s="26" t="s">
         <v>36</v>
       </c>
-      <c r="B23" s="31" t="s">
+      <c r="B23" s="27" t="s">
         <v>175</v>
       </c>
-      <c r="C23" s="31" t="s">
+      <c r="C23" s="27" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="45" x14ac:dyDescent="0.2">
-      <c r="A24" s="28" t="s">
+      <c r="A24" s="24" t="s">
         <v>165</v>
       </c>
-      <c r="B24" s="29" t="s">
+      <c r="B24" s="25" t="s">
         <v>176</v>
       </c>
-      <c r="C24" s="29" t="s">
+      <c r="C24" s="25" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A25" s="30" t="s">
+      <c r="A25" s="26" t="s">
         <v>163</v>
       </c>
-      <c r="B25" s="31" t="s">
+      <c r="B25" s="27" t="s">
         <v>178</v>
       </c>
-      <c r="C25" s="31" t="s">
+      <c r="C25" s="27" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A26" s="28" t="s">
+      <c r="A26" s="24" t="s">
         <v>164</v>
       </c>
-      <c r="B26" s="29" t="s">
+      <c r="B26" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="C26" s="29" t="s">
+      <c r="C26" s="25" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="45" x14ac:dyDescent="0.2">
-      <c r="A27" s="30" t="s">
+      <c r="A27" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="B27" s="31" t="s">
+      <c r="B27" s="27" t="s">
         <v>183</v>
       </c>
-      <c r="C27" s="31" t="s">
+      <c r="C27" s="27" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="38"/>
-      <c r="B28" s="38"/>
-      <c r="C28" s="38"/>
+      <c r="A28" s="35"/>
+      <c r="B28" s="35"/>
+      <c r="C28" s="35"/>
     </row>
     <row r="29" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A29" s="37" t="s">
+      <c r="A29" s="36" t="s">
         <v>39</v>
       </c>
-      <c r="B29" s="37"/>
-      <c r="C29" s="37"/>
+      <c r="B29" s="36"/>
+      <c r="C29" s="36"/>
     </row>
     <row r="30" spans="1:3" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="27" t="s">
+      <c r="A30" s="23" t="s">
         <v>40</v>
       </c>
-      <c r="B30" s="27" t="s">
+      <c r="B30" s="23" t="s">
         <v>41</v>
       </c>
-      <c r="C30" s="27" t="s">
+      <c r="C30" s="23" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A31" s="28" t="s">
+      <c r="A31" s="24" t="s">
         <v>43</v>
       </c>
-      <c r="B31" s="29" t="s">
+      <c r="B31" s="25" t="s">
         <v>44</v>
       </c>
-      <c r="C31" s="29" t="s">
+      <c r="C31" s="25" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A32" s="30" t="s">
+      <c r="A32" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="B32" s="31" t="s">
+      <c r="B32" s="27" t="s">
         <v>47</v>
       </c>
-      <c r="C32" s="31" t="s">
+      <c r="C32" s="27" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A33" s="28" t="s">
+      <c r="A33" s="24" t="s">
         <v>48</v>
       </c>
-      <c r="B33" s="29" t="s">
+      <c r="B33" s="25" t="s">
         <v>49</v>
       </c>
-      <c r="C33" s="29" t="s">
+      <c r="C33" s="25" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A34" s="30" t="s">
+      <c r="A34" s="26" t="s">
         <v>50</v>
       </c>
-      <c r="B34" s="31" t="s">
+      <c r="B34" s="27" t="s">
         <v>51</v>
       </c>
-      <c r="C34" s="31" t="s">
+      <c r="C34" s="27" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A35" s="28" t="s">
+      <c r="A35" s="24" t="s">
         <v>52</v>
       </c>
-      <c r="B35" s="29" t="s">
+      <c r="B35" s="25" t="s">
         <v>53</v>
       </c>
-      <c r="C35" s="29" t="s">
+      <c r="C35" s="25" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A36" s="30" t="s">
+      <c r="A36" s="26" t="s">
         <v>54</v>
       </c>
-      <c r="B36" s="31" t="s">
+      <c r="B36" s="27" t="s">
         <v>55</v>
       </c>
-      <c r="C36" s="31" t="s">
+      <c r="C36" s="27" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A37" s="28" t="s">
+      <c r="A37" s="24" t="s">
         <v>56</v>
       </c>
-      <c r="B37" s="29" t="s">
+      <c r="B37" s="25" t="s">
         <v>57</v>
       </c>
-      <c r="C37" s="29" t="s">
+      <c r="C37" s="25" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A38" s="30" t="s">
+      <c r="A38" s="26" t="s">
         <v>58</v>
       </c>
-      <c r="B38" s="31" t="s">
+      <c r="B38" s="27" t="s">
         <v>59</v>
       </c>
-      <c r="C38" s="31" t="s">
+      <c r="C38" s="27" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A39" s="28" t="s">
+      <c r="A39" s="24" t="s">
         <v>60</v>
       </c>
-      <c r="B39" s="29" t="s">
+      <c r="B39" s="25" t="s">
         <v>61</v>
       </c>
-      <c r="C39" s="29" t="s">
+      <c r="C39" s="25" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A40" s="30" t="s">
+      <c r="A40" s="26" t="s">
         <v>62</v>
       </c>
-      <c r="B40" s="31" t="s">
+      <c r="B40" s="27" t="s">
         <v>63</v>
       </c>
-      <c r="C40" s="31" t="s">
+      <c r="C40" s="27" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A41" s="28" t="s">
+      <c r="A41" s="24" t="s">
         <v>64</v>
       </c>
-      <c r="B41" s="29" t="s">
+      <c r="B41" s="25" t="s">
         <v>65</v>
       </c>
-      <c r="C41" s="29" t="s">
+      <c r="C41" s="25" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A42" s="30" t="s">
+      <c r="A42" s="26" t="s">
         <v>66</v>
       </c>
-      <c r="B42" s="31" t="s">
+      <c r="B42" s="27" t="s">
         <v>67</v>
       </c>
-      <c r="C42" s="31" t="s">
+      <c r="C42" s="27" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A43" s="28" t="s">
+      <c r="A43" s="24" t="s">
         <v>68</v>
       </c>
-      <c r="B43" s="29" t="s">
+      <c r="B43" s="25" t="s">
         <v>69</v>
       </c>
-      <c r="C43" s="29" t="s">
+      <c r="C43" s="25" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A44" s="30" t="s">
+      <c r="A44" s="26" t="s">
         <v>70</v>
       </c>
-      <c r="B44" s="31" t="s">
+      <c r="B44" s="27" t="s">
         <v>71</v>
       </c>
-      <c r="C44" s="31" t="s">
+      <c r="C44" s="27" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A45" s="28" t="s">
+      <c r="A45" s="24" t="s">
         <v>72</v>
       </c>
-      <c r="B45" s="29" t="s">
+      <c r="B45" s="25" t="s">
         <v>73</v>
       </c>
-      <c r="C45" s="29" t="s">
+      <c r="C45" s="25" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A46" s="30" t="s">
+      <c r="A46" s="26" t="s">
         <v>74</v>
       </c>
-      <c r="B46" s="31" t="s">
+      <c r="B46" s="27" t="s">
         <v>75</v>
       </c>
-      <c r="C46" s="31" t="s">
+      <c r="C46" s="27" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A47" s="28" t="s">
+      <c r="A47" s="24" t="s">
         <v>77</v>
       </c>
-      <c r="B47" s="29" t="s">
+      <c r="B47" s="25" t="s">
         <v>78</v>
       </c>
-      <c r="C47" s="29" t="s">
+      <c r="C47" s="25" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A48" s="30" t="s">
+      <c r="A48" s="26" t="s">
         <v>80</v>
       </c>
-      <c r="B48" s="31" t="s">
+      <c r="B48" s="27" t="s">
         <v>81</v>
       </c>
-      <c r="C48" s="31" t="s">
+      <c r="C48" s="27" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="49" spans="1:3" ht="60" x14ac:dyDescent="0.2">
-      <c r="A49" s="28" t="s">
+      <c r="A49" s="24" t="s">
         <v>83</v>
       </c>
-      <c r="B49" s="29" t="s">
+      <c r="B49" s="25" t="s">
         <v>179</v>
       </c>
-      <c r="C49" s="29" t="s">
+      <c r="C49" s="25" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="50" spans="1:3" ht="45" x14ac:dyDescent="0.2">
-      <c r="A50" s="30" t="s">
+    <row r="50" spans="1:3" ht="75" x14ac:dyDescent="0.2">
+      <c r="A50" s="26" t="s">
         <v>84</v>
       </c>
-      <c r="B50" s="31" t="s">
+      <c r="B50" s="27" t="s">
         <v>158</v>
       </c>
-      <c r="C50" s="31" t="s">
-        <v>45</v>
+      <c r="C50" s="27" t="s">
+        <v>186</v>
       </c>
     </row>
     <row r="51" spans="1:3" ht="75" x14ac:dyDescent="0.2">
-      <c r="A51" s="28" t="s">
+      <c r="A51" s="24" t="s">
         <v>85</v>
       </c>
-      <c r="B51" s="29" t="s">
+      <c r="B51" s="25" t="s">
         <v>185</v>
       </c>
-      <c r="C51" s="29" t="s">
+      <c r="C51" s="25" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="52" spans="1:3" ht="30" x14ac:dyDescent="0.2">
-      <c r="A52" s="30" t="s">
+      <c r="A52" s="26" t="s">
         <v>87</v>
       </c>
-      <c r="B52" s="31" t="s">
+      <c r="B52" s="27" t="s">
         <v>88</v>
       </c>
-      <c r="C52" s="31" t="s">
+      <c r="C52" s="27" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="53" spans="1:3" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="38"/>
-      <c r="B53" s="38"/>
-      <c r="C53" s="38"/>
+      <c r="A53" s="35"/>
+      <c r="B53" s="35"/>
+      <c r="C53" s="35"/>
     </row>
     <row r="54" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A54" s="37" t="s">
+      <c r="A54" s="36" t="s">
         <v>90</v>
       </c>
-      <c r="B54" s="37"/>
-      <c r="C54" s="37"/>
+      <c r="B54" s="36"/>
+      <c r="C54" s="36"/>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A55" s="32" t="s">
+      <c r="A55" s="28" t="s">
         <v>91</v>
       </c>
-      <c r="B55" s="39" t="s">
+      <c r="B55" s="45" t="s">
         <v>92</v>
       </c>
-      <c r="C55" s="40"/>
+      <c r="C55" s="46"/>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A56" s="32" t="s">
+      <c r="A56" s="28" t="s">
         <v>91</v>
       </c>
-      <c r="B56" s="41" t="s">
+      <c r="B56" s="33" t="s">
         <v>180</v>
       </c>
-      <c r="C56" s="42"/>
+      <c r="C56" s="34"/>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A57" s="32" t="s">
+      <c r="A57" s="28" t="s">
         <v>91</v>
       </c>
-      <c r="B57" s="41" t="s">
+      <c r="B57" s="33" t="s">
         <v>93</v>
       </c>
-      <c r="C57" s="42"/>
+      <c r="C57" s="34"/>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A58" s="32" t="s">
+      <c r="A58" s="28" t="s">
         <v>91</v>
       </c>
-      <c r="B58" s="41" t="s">
+      <c r="B58" s="33" t="s">
         <v>94</v>
       </c>
-      <c r="C58" s="42"/>
+      <c r="C58" s="34"/>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A59" s="32" t="s">
+      <c r="A59" s="28" t="s">
         <v>91</v>
       </c>
-      <c r="B59" s="41" t="s">
+      <c r="B59" s="33" t="s">
         <v>95</v>
       </c>
-      <c r="C59" s="42"/>
+      <c r="C59" s="34"/>
     </row>
     <row r="60" spans="1:3" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="38"/>
-      <c r="B60" s="38"/>
-      <c r="C60" s="38"/>
+      <c r="A60" s="35"/>
+      <c r="B60" s="35"/>
+      <c r="C60" s="35"/>
     </row>
     <row r="61" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A61" s="37" t="s">
+      <c r="A61" s="36" t="s">
         <v>96</v>
       </c>
-      <c r="B61" s="37"/>
-      <c r="C61" s="37"/>
+      <c r="B61" s="36"/>
+      <c r="C61" s="36"/>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A62" s="32" t="s">
+      <c r="A62" s="28" t="s">
         <v>91</v>
       </c>
-      <c r="B62" s="39" t="s">
+      <c r="B62" s="45" t="s">
         <v>97</v>
       </c>
-      <c r="C62" s="40"/>
+      <c r="C62" s="46"/>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A63" s="32" t="s">
+      <c r="A63" s="28" t="s">
         <v>91</v>
       </c>
-      <c r="B63" s="41" t="s">
+      <c r="B63" s="33" t="s">
         <v>98</v>
       </c>
-      <c r="C63" s="42"/>
+      <c r="C63" s="34"/>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A64" s="32" t="s">
+      <c r="A64" s="28" t="s">
         <v>91</v>
       </c>
-      <c r="B64" s="41" t="s">
+      <c r="B64" s="33" t="s">
         <v>99</v>
       </c>
-      <c r="C64" s="42"/>
+      <c r="C64" s="34"/>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A65" s="32" t="s">
+      <c r="A65" s="28" t="s">
         <v>91</v>
       </c>
-      <c r="B65" s="41" t="s">
+      <c r="B65" s="33" t="s">
         <v>182</v>
       </c>
-      <c r="C65" s="42"/>
+      <c r="C65" s="34"/>
     </row>
     <row r="66" spans="1:3" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="38"/>
-      <c r="B66" s="38"/>
-      <c r="C66" s="38"/>
+      <c r="A66" s="35"/>
+      <c r="B66" s="35"/>
+      <c r="C66" s="35"/>
     </row>
     <row r="67" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A67" s="37" t="s">
+      <c r="A67" s="36" t="s">
         <v>100</v>
       </c>
-      <c r="B67" s="37"/>
-      <c r="C67" s="37"/>
+      <c r="B67" s="36"/>
+      <c r="C67" s="36"/>
     </row>
     <row r="68" spans="1:3" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="27" t="s">
+      <c r="A68" s="23" t="s">
         <v>101</v>
       </c>
-      <c r="B68" s="27" t="s">
+      <c r="B68" s="23" t="s">
         <v>102</v>
       </c>
-      <c r="C68" s="27"/>
+      <c r="C68" s="23"/>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A69" s="28" t="s">
+      <c r="A69" s="24" t="s">
         <v>159</v>
       </c>
-      <c r="B69" s="29" t="s">
+      <c r="B69" s="25" t="s">
         <v>103</v>
       </c>
-      <c r="C69" s="29"/>
+      <c r="C69" s="25"/>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A70" s="30" t="s">
+      <c r="A70" s="26" t="s">
         <v>104</v>
       </c>
-      <c r="B70" s="31" t="s">
+      <c r="B70" s="27" t="s">
         <v>105</v>
       </c>
-      <c r="C70" s="31"/>
+      <c r="C70" s="27"/>
     </row>
     <row r="71" spans="1:3" ht="60" x14ac:dyDescent="0.2">
-      <c r="A71" s="30" t="s">
+      <c r="A71" s="26" t="s">
         <v>106</v>
       </c>
-      <c r="B71" s="31" t="s">
+      <c r="B71" s="27" t="s">
         <v>184</v>
       </c>
-      <c r="C71" s="31"/>
+      <c r="C71" s="27"/>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A72" s="43"/>
-      <c r="B72" s="43"/>
-      <c r="C72" s="43"/>
+      <c r="A72" s="32"/>
+      <c r="B72" s="32"/>
+      <c r="C72" s="32"/>
     </row>
     <row r="73" spans="1:3" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="27" t="s">
+      <c r="A73" s="23" t="s">
         <v>107</v>
       </c>
-      <c r="B73" s="44"/>
-      <c r="C73" s="45"/>
+      <c r="B73" s="39"/>
+      <c r="C73" s="40"/>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A74" s="32"/>
-      <c r="B74" s="46" t="s">
+      <c r="A74" s="28"/>
+      <c r="B74" s="41" t="s">
         <v>108</v>
       </c>
-      <c r="C74" s="47"/>
+      <c r="C74" s="42"/>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A75" s="32"/>
-      <c r="B75" s="48" t="s">
+      <c r="A75" s="28"/>
+      <c r="B75" s="43" t="s">
         <v>109</v>
       </c>
-      <c r="C75" s="49"/>
+      <c r="C75" s="44"/>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A76" s="32"/>
-      <c r="B76" s="48" t="s">
+      <c r="A76" s="28"/>
+      <c r="B76" s="43" t="s">
         <v>110</v>
       </c>
-      <c r="C76" s="49"/>
+      <c r="C76" s="44"/>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A77" s="32"/>
-      <c r="B77" s="48" t="s">
+      <c r="A77" s="28"/>
+      <c r="B77" s="43" t="s">
         <v>111</v>
       </c>
-      <c r="C77" s="49"/>
+      <c r="C77" s="44"/>
     </row>
     <row r="78" spans="1:3" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A78" s="38"/>
-      <c r="B78" s="38"/>
-      <c r="C78" s="38"/>
+      <c r="A78" s="35"/>
+      <c r="B78" s="35"/>
+      <c r="C78" s="35"/>
     </row>
     <row r="79" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A79" s="37" t="s">
+      <c r="A79" s="36" t="s">
         <v>177</v>
       </c>
-      <c r="B79" s="37"/>
-      <c r="C79" s="37"/>
+      <c r="B79" s="36"/>
+      <c r="C79" s="36"/>
     </row>
     <row r="80" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A80" s="33" t="s">
+      <c r="A80" s="29" t="s">
         <v>112</v>
       </c>
-      <c r="B80" s="50" t="s">
+      <c r="B80" s="37" t="s">
         <v>113</v>
       </c>
-      <c r="C80" s="51"/>
+      <c r="C80" s="38"/>
     </row>
     <row r="81" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A81" s="33" t="s">
+      <c r="A81" s="29" t="s">
         <v>112</v>
       </c>
-      <c r="B81" s="52" t="s">
+      <c r="B81" s="30" t="s">
         <v>114</v>
       </c>
-      <c r="C81" s="53"/>
+      <c r="C81" s="31"/>
     </row>
     <row r="82" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A82" s="33" t="s">
+      <c r="A82" s="29" t="s">
         <v>112</v>
       </c>
-      <c r="B82" s="52" t="s">
+      <c r="B82" s="30" t="s">
         <v>115</v>
       </c>
-      <c r="C82" s="53"/>
+      <c r="C82" s="31"/>
     </row>
     <row r="83" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A83" s="33" t="s">
+      <c r="A83" s="29" t="s">
         <v>112</v>
       </c>
-      <c r="B83" s="52" t="s">
+      <c r="B83" s="30" t="s">
         <v>116</v>
       </c>
-      <c r="C83" s="53"/>
+      <c r="C83" s="31"/>
     </row>
     <row r="84" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A84" s="33" t="s">
+      <c r="A84" s="29" t="s">
         <v>112</v>
       </c>
-      <c r="B84" s="52" t="s">
+      <c r="B84" s="30" t="s">
         <v>181</v>
       </c>
-      <c r="C84" s="53"/>
+      <c r="C84" s="31"/>
     </row>
     <row r="85" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A85" s="33" t="s">
+      <c r="A85" s="29" t="s">
         <v>112</v>
       </c>
-      <c r="B85" s="52" t="s">
+      <c r="B85" s="30" t="s">
         <v>117</v>
       </c>
-      <c r="C85" s="53"/>
+      <c r="C85" s="31"/>
     </row>
     <row r="86" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A86" s="33" t="s">
+      <c r="A86" s="29" t="s">
         <v>112</v>
       </c>
-      <c r="B86" s="52" t="s">
+      <c r="B86" s="30" t="s">
         <v>118</v>
       </c>
-      <c r="C86" s="53"/>
+      <c r="C86" s="31"/>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A87" s="43"/>
-      <c r="B87" s="43"/>
-      <c r="C87" s="43"/>
+      <c r="A87" s="32"/>
+      <c r="B87" s="32"/>
+      <c r="C87" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="41">
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="A60:C60"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="A16:C16"/>
+    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="A29:C29"/>
+    <mergeCell ref="A53:C53"/>
+    <mergeCell ref="A54:C54"/>
+    <mergeCell ref="B55:C55"/>
+    <mergeCell ref="B56:C56"/>
+    <mergeCell ref="B57:C57"/>
+    <mergeCell ref="B58:C58"/>
+    <mergeCell ref="B59:C59"/>
+    <mergeCell ref="B77:C77"/>
+    <mergeCell ref="A61:C61"/>
+    <mergeCell ref="B62:C62"/>
+    <mergeCell ref="B63:C63"/>
+    <mergeCell ref="B64:C64"/>
+    <mergeCell ref="A66:C66"/>
+    <mergeCell ref="A67:C67"/>
     <mergeCell ref="B84:C84"/>
     <mergeCell ref="B85:C85"/>
     <mergeCell ref="B86:C86"/>
@@ -2493,31 +2521,6 @@
     <mergeCell ref="B74:C74"/>
     <mergeCell ref="B75:C75"/>
     <mergeCell ref="B76:C76"/>
-    <mergeCell ref="B77:C77"/>
-    <mergeCell ref="A61:C61"/>
-    <mergeCell ref="B62:C62"/>
-    <mergeCell ref="B63:C63"/>
-    <mergeCell ref="B64:C64"/>
-    <mergeCell ref="A66:C66"/>
-    <mergeCell ref="A67:C67"/>
-    <mergeCell ref="B55:C55"/>
-    <mergeCell ref="B56:C56"/>
-    <mergeCell ref="B57:C57"/>
-    <mergeCell ref="B58:C58"/>
-    <mergeCell ref="B59:C59"/>
-    <mergeCell ref="A60:C60"/>
-    <mergeCell ref="A15:C15"/>
-    <mergeCell ref="A16:C16"/>
-    <mergeCell ref="A28:C28"/>
-    <mergeCell ref="A29:C29"/>
-    <mergeCell ref="A53:C53"/>
-    <mergeCell ref="A54:C54"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="A9:C9"/>
-    <mergeCell ref="A10:C10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -2544,50 +2547,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="51" t="s">
         <v>119</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
-      <c r="I1" s="8"/>
-      <c r="J1" s="9"/>
+      <c r="B1" s="52"/>
+      <c r="C1" s="52"/>
+      <c r="D1" s="52"/>
+      <c r="E1" s="52"/>
+      <c r="F1" s="52"/>
+      <c r="G1" s="52"/>
+      <c r="H1" s="52"/>
+      <c r="I1" s="52"/>
+      <c r="J1" s="53"/>
     </row>
     <row r="2" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="50" t="s">
         <v>120</v>
       </c>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="6"/>
-      <c r="H2" s="6"/>
-      <c r="I2" s="6"/>
-      <c r="J2" s="6"/>
+      <c r="C2" s="50"/>
+      <c r="D2" s="50"/>
+      <c r="E2" s="50"/>
+      <c r="F2" s="50"/>
+      <c r="G2" s="50"/>
+      <c r="H2" s="50"/>
+      <c r="I2" s="50"/>
+      <c r="J2" s="50"/>
     </row>
     <row r="3" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="50" t="s">
         <v>122</v>
       </c>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
-      <c r="E3" s="6"/>
-      <c r="F3" s="6"/>
-      <c r="G3" s="6"/>
-      <c r="H3" s="6"/>
-      <c r="I3" s="6"/>
-      <c r="J3" s="6"/>
+      <c r="C3" s="50"/>
+      <c r="D3" s="50"/>
+      <c r="E3" s="50"/>
+      <c r="F3" s="50"/>
+      <c r="G3" s="50"/>
+      <c r="H3" s="50"/>
+      <c r="I3" s="50"/>
+      <c r="J3" s="50"/>
     </row>
     <row r="4" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
@@ -2844,10 +2847,10 @@
       <c r="J14" s="3"/>
     </row>
     <row r="15" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A15" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="B15" s="10" t="s">
+      <c r="A15" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B15" s="6" t="s">
         <v>60</v>
       </c>
       <c r="C15" s="3"/>
@@ -2866,10 +2869,10 @@
       <c r="J15" s="3"/>
     </row>
     <row r="16" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A16" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="B16" s="10" t="s">
+      <c r="A16" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B16" s="6" t="s">
         <v>62</v>
       </c>
       <c r="C16" s="3"/>
@@ -2888,10 +2891,10 @@
       <c r="J16" s="3"/>
     </row>
     <row r="17" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A17" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="B17" s="10" t="s">
+      <c r="A17" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B17" s="6" t="s">
         <v>64</v>
       </c>
       <c r="C17" s="3"/>
@@ -2910,10 +2913,10 @@
       <c r="J17" s="3"/>
     </row>
     <row r="18" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A18" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="B18" s="10" t="s">
+      <c r="A18" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B18" s="6" t="s">
         <v>66</v>
       </c>
       <c r="C18" s="3"/>
@@ -2932,10 +2935,10 @@
       <c r="J18" s="3"/>
     </row>
     <row r="19" spans="1:10" ht="32" x14ac:dyDescent="0.2">
-      <c r="A19" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="B19" s="10" t="s">
+      <c r="A19" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B19" s="6" t="s">
         <v>87</v>
       </c>
       <c r="C19" s="3" t="s">
@@ -2954,15 +2957,15 @@
       <c r="J19" s="3"/>
     </row>
     <row r="20" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A20" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="B20" s="10" t="s">
+      <c r="A20" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B20" s="6" t="s">
         <v>70</v>
       </c>
       <c r="C20" s="3"/>
-      <c r="D20" s="11"/>
-      <c r="E20" s="10" t="s">
+      <c r="D20" s="7"/>
+      <c r="E20" s="6" t="s">
         <v>70</v>
       </c>
       <c r="F20" s="3" t="s">
@@ -2980,7 +2983,7 @@
       <c r="B21" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="C21" s="24" t="s">
+      <c r="C21" s="20" t="s">
         <v>135</v>
       </c>
       <c r="D21" s="3"/>
@@ -2990,7 +2993,7 @@
       <c r="F21" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="G21" s="25">
+      <c r="G21" s="21">
         <v>1</v>
       </c>
       <c r="H21" s="3"/>
@@ -3004,7 +3007,7 @@
       <c r="B22" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="C22" s="24" t="s">
+      <c r="C22" s="20" t="s">
         <v>137</v>
       </c>
       <c r="D22" s="3"/>
@@ -3014,7 +3017,7 @@
       <c r="F22" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="G22" s="26">
+      <c r="G22" s="22">
         <v>1</v>
       </c>
       <c r="H22" s="3"/>
@@ -3022,15 +3025,15 @@
       <c r="J22" s="3"/>
     </row>
     <row r="23" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A23" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="B23" s="10" t="s">
+      <c r="A23" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B23" s="6" t="s">
         <v>72</v>
       </c>
       <c r="C23" s="3"/>
-      <c r="D23" s="12"/>
-      <c r="E23" s="10" t="s">
+      <c r="D23" s="8"/>
+      <c r="E23" s="6" t="s">
         <v>139</v>
       </c>
       <c r="F23" s="3" t="s">
@@ -3044,21 +3047,21 @@
       <c r="J23" s="3"/>
     </row>
     <row r="24" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A24" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="B24" s="10" t="s">
+      <c r="A24" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B24" s="6" t="s">
         <v>48</v>
       </c>
       <c r="C24" s="3"/>
-      <c r="D24" s="12" t="b">
+      <c r="D24" s="8" t="b">
         <f>EXACT(G5,"Option 1")</f>
         <v>1</v>
       </c>
-      <c r="E24" s="14" t="s">
+      <c r="E24" s="10" t="s">
         <v>141</v>
       </c>
-      <c r="F24" s="10" t="s">
+      <c r="F24" s="6" t="s">
         <v>7</v>
       </c>
       <c r="G24" s="3" t="s">
@@ -3069,338 +3072,338 @@
       <c r="J24" s="3"/>
     </row>
     <row r="25" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A25" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="B25" s="14" t="s">
+      <c r="A25" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B25" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="C25" s="14"/>
-      <c r="D25" s="20" t="b">
+      <c r="C25" s="10"/>
+      <c r="D25" s="16" t="b">
         <f>NOT(EXACT(G5,"Option 1"))</f>
         <v>0</v>
       </c>
-      <c r="E25" s="14" t="s">
+      <c r="E25" s="10" t="s">
         <v>142</v>
       </c>
-      <c r="F25" s="14" t="s">
-        <v>7</v>
-      </c>
-      <c r="G25" s="14" t="s">
+      <c r="F25" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="G25" s="10" t="s">
         <v>124</v>
       </c>
-      <c r="H25" s="14"/>
-      <c r="I25" s="14"/>
-      <c r="J25" s="14"/>
+      <c r="H25" s="10"/>
+      <c r="I25" s="10"/>
+      <c r="J25" s="10"/>
     </row>
     <row r="26" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A26" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="B26" s="15" t="s">
+      <c r="A26" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B26" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="C26" s="15"/>
-      <c r="D26" s="18" t="s">
-        <v>7</v>
-      </c>
-      <c r="E26" s="15" t="s">
+      <c r="C26" s="11"/>
+      <c r="D26" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="E26" s="11" t="s">
         <v>143</v>
       </c>
-      <c r="F26" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="G26" s="15" t="s">
+      <c r="F26" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="G26" s="11" t="s">
         <v>124</v>
       </c>
-      <c r="H26" s="15"/>
-      <c r="I26" s="15"/>
-      <c r="J26" s="15"/>
+      <c r="H26" s="11"/>
+      <c r="I26" s="11"/>
+      <c r="J26" s="11"/>
     </row>
     <row r="27" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A27" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="B27" s="15" t="s">
+      <c r="A27" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B27" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="C27" s="15" t="s">
+      <c r="C27" s="11" t="s">
         <v>144</v>
       </c>
-      <c r="D27" s="18"/>
-      <c r="E27" s="15" t="s">
+      <c r="D27" s="14"/>
+      <c r="E27" s="11" t="s">
         <v>145</v>
       </c>
-      <c r="F27" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="G27" s="15">
+      <c r="F27" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="G27" s="11">
         <f>G6+G7</f>
         <v>2</v>
       </c>
-      <c r="H27" s="15"/>
-      <c r="I27" s="15"/>
-      <c r="J27" s="15"/>
+      <c r="H27" s="11"/>
+      <c r="I27" s="11"/>
+      <c r="J27" s="11"/>
     </row>
     <row r="28" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A28" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="B28" s="15" t="s">
+      <c r="A28" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B28" s="11" t="s">
         <v>84</v>
       </c>
-      <c r="C28" s="15" t="s">
+      <c r="C28" s="11" t="s">
         <v>162</v>
       </c>
-      <c r="D28" s="18"/>
-      <c r="E28" s="15" t="s">
+      <c r="D28" s="14"/>
+      <c r="E28" s="11" t="s">
         <v>168</v>
       </c>
-      <c r="F28" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="G28" s="15"/>
-      <c r="H28" s="15"/>
-      <c r="I28" s="15"/>
-      <c r="J28" s="15"/>
+      <c r="F28" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="G28" s="11"/>
+      <c r="H28" s="11"/>
+      <c r="I28" s="11"/>
+      <c r="J28" s="11"/>
     </row>
     <row r="29" spans="1:10" ht="16" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="B29" s="16" t="s">
+      <c r="A29" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B29" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="C29" s="16"/>
-      <c r="D29" s="19"/>
-      <c r="E29" s="16" t="s">
+      <c r="C29" s="12"/>
+      <c r="D29" s="15"/>
+      <c r="E29" s="12" t="s">
         <v>146</v>
       </c>
-      <c r="F29" s="16" t="s">
-        <v>7</v>
-      </c>
-      <c r="G29" s="16" t="s">
+      <c r="F29" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="G29" s="12" t="s">
         <v>147</v>
       </c>
-      <c r="H29" s="16"/>
-      <c r="I29" s="16"/>
-      <c r="J29" s="16"/>
+      <c r="H29" s="12"/>
+      <c r="I29" s="12"/>
+      <c r="J29" s="12"/>
     </row>
     <row r="30" spans="1:10" ht="16" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="13" t="s">
+      <c r="A30" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="B30" s="16" t="s">
+      <c r="B30" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="C30" s="16"/>
-      <c r="D30" s="19"/>
-      <c r="E30" s="16" t="s">
+      <c r="C30" s="12"/>
+      <c r="D30" s="15"/>
+      <c r="E30" s="12" t="s">
         <v>148</v>
       </c>
-      <c r="F30" s="16" t="s">
+      <c r="F30" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="G30" s="16">
+      <c r="G30" s="12">
         <v>1</v>
       </c>
-      <c r="H30" s="16"/>
-      <c r="I30" s="16"/>
-      <c r="J30" s="16"/>
+      <c r="H30" s="12"/>
+      <c r="I30" s="12"/>
+      <c r="J30" s="12"/>
     </row>
     <row r="31" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A31" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="B31" s="15" t="s">
+      <c r="A31" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B31" s="11" t="s">
         <v>84</v>
       </c>
-      <c r="C31" s="17" t="s">
+      <c r="C31" s="13" t="s">
         <v>162</v>
       </c>
-      <c r="D31" s="18"/>
-      <c r="E31" s="15" t="s">
+      <c r="D31" s="14"/>
+      <c r="E31" s="11" t="s">
         <v>169</v>
       </c>
-      <c r="F31" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="G31" s="15"/>
-      <c r="H31" s="15"/>
-      <c r="I31" s="15"/>
-      <c r="J31" s="15"/>
+      <c r="F31" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="G31" s="11"/>
+      <c r="H31" s="11"/>
+      <c r="I31" s="11"/>
+      <c r="J31" s="11"/>
     </row>
     <row r="32" spans="1:10" ht="16" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="B32" s="16" t="s">
+      <c r="A32" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B32" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="C32" s="16"/>
-      <c r="D32" s="19"/>
-      <c r="E32" s="16" t="s">
+      <c r="C32" s="12"/>
+      <c r="D32" s="15"/>
+      <c r="E32" s="12" t="s">
         <v>146</v>
       </c>
-      <c r="F32" s="16" t="s">
-        <v>7</v>
-      </c>
-      <c r="G32" s="16" t="s">
+      <c r="F32" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="G32" s="12" t="s">
         <v>147</v>
       </c>
-      <c r="H32" s="16"/>
-      <c r="I32" s="16"/>
-      <c r="J32" s="16"/>
+      <c r="H32" s="12"/>
+      <c r="I32" s="12"/>
+      <c r="J32" s="12"/>
     </row>
     <row r="33" spans="1:10" ht="16" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="13" t="s">
+      <c r="A33" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="B33" s="16" t="s">
+      <c r="B33" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="C33" s="16"/>
-      <c r="D33" s="19"/>
-      <c r="E33" s="16" t="s">
+      <c r="C33" s="12"/>
+      <c r="D33" s="15"/>
+      <c r="E33" s="12" t="s">
         <v>148</v>
       </c>
-      <c r="F33" s="16" t="s">
+      <c r="F33" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="G33" s="16">
+      <c r="G33" s="12">
         <v>1</v>
       </c>
-      <c r="H33" s="16"/>
-      <c r="I33" s="16"/>
-      <c r="J33" s="16"/>
+      <c r="H33" s="12"/>
+      <c r="I33" s="12"/>
+      <c r="J33" s="12"/>
     </row>
     <row r="34" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A34" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="B34" s="15" t="s">
+      <c r="A34" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B34" s="11" t="s">
         <v>84</v>
       </c>
-      <c r="C34" s="17" t="s">
+      <c r="C34" s="13" t="s">
         <v>161</v>
       </c>
-      <c r="D34" s="18"/>
-      <c r="E34" s="15" t="s">
+      <c r="D34" s="14"/>
+      <c r="E34" s="11" t="s">
         <v>170</v>
       </c>
-      <c r="F34" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="G34" s="15"/>
-      <c r="H34" s="15"/>
-      <c r="I34" s="15"/>
-      <c r="J34" s="15"/>
+      <c r="F34" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="G34" s="11"/>
+      <c r="H34" s="11"/>
+      <c r="I34" s="11"/>
+      <c r="J34" s="11"/>
     </row>
     <row r="35" spans="1:10" ht="16" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="B35" s="16" t="s">
+      <c r="A35" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B35" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="C35" s="16"/>
-      <c r="D35" s="19"/>
-      <c r="E35" s="16" t="s">
+      <c r="C35" s="12"/>
+      <c r="D35" s="15"/>
+      <c r="E35" s="12" t="s">
         <v>146</v>
       </c>
-      <c r="F35" s="16" t="s">
-        <v>7</v>
-      </c>
-      <c r="G35" s="16" t="s">
+      <c r="F35" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="G35" s="12" t="s">
         <v>147</v>
       </c>
-      <c r="H35" s="16"/>
-      <c r="I35" s="16"/>
-      <c r="J35" s="16"/>
+      <c r="H35" s="12"/>
+      <c r="I35" s="12"/>
+      <c r="J35" s="12"/>
     </row>
     <row r="36" spans="1:10" ht="16" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="19" t="s">
+      <c r="A36" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="B36" s="16" t="s">
+      <c r="B36" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="C36" s="16"/>
-      <c r="D36" s="19"/>
-      <c r="E36" s="16" t="s">
+      <c r="C36" s="12"/>
+      <c r="D36" s="15"/>
+      <c r="E36" s="12" t="s">
         <v>166</v>
       </c>
-      <c r="F36" s="16"/>
-      <c r="G36" s="16"/>
-      <c r="H36" s="16"/>
-      <c r="I36" s="16"/>
-      <c r="J36" s="16"/>
+      <c r="F36" s="12"/>
+      <c r="G36" s="12"/>
+      <c r="H36" s="12"/>
+      <c r="I36" s="12"/>
+      <c r="J36" s="12"/>
     </row>
     <row r="37" spans="1:10" ht="16" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="B37" s="15" t="s">
+      <c r="A37" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B37" s="11" t="s">
         <v>84</v>
       </c>
-      <c r="C37" s="17" t="s">
+      <c r="C37" s="13" t="s">
         <v>162</v>
       </c>
-      <c r="D37" s="18"/>
-      <c r="E37" s="15" t="s">
+      <c r="D37" s="14"/>
+      <c r="E37" s="11" t="s">
         <v>171</v>
       </c>
-      <c r="F37" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="G37" s="15"/>
-      <c r="H37" s="15"/>
-      <c r="I37" s="15"/>
-      <c r="J37" s="15"/>
+      <c r="F37" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="G37" s="11"/>
+      <c r="H37" s="11"/>
+      <c r="I37" s="11"/>
+      <c r="J37" s="11"/>
     </row>
     <row r="38" spans="1:10" ht="16" outlineLevel="2" x14ac:dyDescent="0.2">
-      <c r="A38" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="B38" s="16" t="s">
+      <c r="A38" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B38" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="C38" s="16"/>
-      <c r="D38" s="19"/>
-      <c r="E38" s="16" t="s">
+      <c r="C38" s="12"/>
+      <c r="D38" s="15"/>
+      <c r="E38" s="12" t="s">
         <v>146</v>
       </c>
-      <c r="F38" s="16" t="s">
-        <v>7</v>
-      </c>
-      <c r="G38" s="16" t="s">
+      <c r="F38" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="G38" s="12" t="s">
         <v>147</v>
       </c>
-      <c r="H38" s="16"/>
-      <c r="I38" s="16"/>
-      <c r="J38" s="16"/>
+      <c r="H38" s="12"/>
+      <c r="I38" s="12"/>
+      <c r="J38" s="12"/>
     </row>
     <row r="39" spans="1:10" ht="16" outlineLevel="2" x14ac:dyDescent="0.2">
-      <c r="A39" s="21" t="s">
+      <c r="A39" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="B39" s="22" t="s">
+      <c r="B39" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="C39" s="22"/>
-      <c r="D39" s="23"/>
-      <c r="E39" s="22" t="s">
+      <c r="C39" s="18"/>
+      <c r="D39" s="19"/>
+      <c r="E39" s="18" t="s">
         <v>148</v>
       </c>
-      <c r="F39" s="22" t="s">
+      <c r="F39" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="G39" s="22">
+      <c r="G39" s="18">
         <v>1</v>
       </c>
-      <c r="H39" s="22"/>
-      <c r="I39" s="22"/>
-      <c r="J39" s="22"/>
+      <c r="H39" s="18"/>
+      <c r="I39" s="18"/>
+      <c r="J39" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>

<commit_message>
fix: teach Enum Parameter contract in the Excel schema template README
</commit_message>
<xml_diff>
--- a/guardian-service/artifacts/template.xlsx
+++ b/guardian-service/artifacts/template.xlsx
@@ -1496,7 +1496,7 @@
       </c>
       <c r="B20" s="25" t="inlineStr">
         <is>
-          <t>Type-dependent: unit symbol (Prefix/Postfix), regex (Pattern), math expression (Auto-Calculate), JSON font object (Help Text), JSON column array (Table), parent field key (Country, State/Province). Blank for all other types.</t>
+          <t>Type-dependent: enum name (Enum), unit symbol (Prefix/Postfix), regex (Pattern), math expression (Auto-Calculate), JSON font object (Help Text), JSON column array (Table), parent field key (Country, State/Province). Blank for all other types.</t>
         </is>
       </c>
       <c r="C20" s="25" t="inlineStr">
@@ -1969,7 +1969,7 @@
       </c>
       <c r="B49" s="25" t="inlineStr">
         <is>
-          <t>Dropdown list — values defined in the Enums tab. The field's Description must match the "Enum Name" column and the schema name (row 1) must match "Schema name" — both case-sensitive.</t>
+          <t>Dropdown list — values defined in the Enums tab. The field's Parameter must exactly match the "Enum Name" column and the schema name (row 1) must match "Schema name" — both case-sensitive.</t>
         </is>
       </c>
       <c r="C49" s="25" t="inlineStr">
@@ -2149,7 +2149,7 @@
       </c>
       <c r="B61" s="33" t="inlineStr">
         <is>
-          <t>The field's Description value must exactly match the "Enum Name" column in the Enums tab, and the schema name (row 1) must exactly match the "Schema name" column (both case-sensitive).</t>
+          <t>The field's Parameter value must exactly match the "Enum Name" column in the Enums tab, and the schema name (row 1) must exactly match the "Schema name" column (both case-sensitive).</t>
         </is>
       </c>
       <c r="C61" s="58" t="n"/>
@@ -2522,7 +2522,6 @@
     <mergeCell ref="A3:C3"/>
     <mergeCell ref="B93:C93"/>
     <mergeCell ref="A2:C2"/>
-    <mergeCell ref="B79:C79"/>
     <mergeCell ref="B70:C70"/>
     <mergeCell ref="A71:C71"/>
     <mergeCell ref="B86:C86"/>
@@ -2533,29 +2532,30 @@
     <mergeCell ref="A4:C4"/>
     <mergeCell ref="B88:C88"/>
     <mergeCell ref="B82:C82"/>
+    <mergeCell ref="A72:C72"/>
     <mergeCell ref="A10:C10"/>
     <mergeCell ref="A28:C28"/>
     <mergeCell ref="B87:C87"/>
-    <mergeCell ref="A72:C72"/>
     <mergeCell ref="B69:C69"/>
     <mergeCell ref="B78:C78"/>
-    <mergeCell ref="A16:C16"/>
     <mergeCell ref="A58:C58"/>
     <mergeCell ref="A9:C9"/>
     <mergeCell ref="A77:C77"/>
     <mergeCell ref="A83:C83"/>
     <mergeCell ref="A15:C15"/>
     <mergeCell ref="A59:C59"/>
+    <mergeCell ref="B92:C92"/>
     <mergeCell ref="B68:C68"/>
-    <mergeCell ref="B92:C92"/>
     <mergeCell ref="B64:C64"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A94:C94"/>
+    <mergeCell ref="B80:C80"/>
     <mergeCell ref="B89:C89"/>
-    <mergeCell ref="B80:C80"/>
     <mergeCell ref="B85:C85"/>
     <mergeCell ref="B63:C63"/>
+    <mergeCell ref="B79:C79"/>
     <mergeCell ref="A65:C65"/>
+    <mergeCell ref="A16:C16"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>